<commit_message>
Update travel sheets and add new snapshots for planning, approved, and reconciled versions
</commit_message>
<xml_diff>
--- a/data/travel_sheet_v3_reconciled.xlsx
+++ b/data/travel_sheet_v3_reconciled.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arezo-o\Downloads\ArezooHassannezhad\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F902DFAC-564A-403E-98EA-C2E4FFE1A395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF9D9D1-B7EF-4C30-9DFF-902202B5101A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -453,13 +453,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -839,7 +838,7 @@
       <c r="J2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="2"/>
+      <c r="K2" s="4"/>
       <c r="L2" s="2" t="s">
         <v>20</v>
       </c>
@@ -875,7 +874,7 @@
       <c r="J3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="2"/>
+      <c r="K3" s="4"/>
       <c r="L3" s="2" t="s">
         <v>20</v>
       </c>
@@ -911,7 +910,7 @@
       <c r="J4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="2"/>
+      <c r="K4" s="4"/>
       <c r="L4" s="2" t="s">
         <v>20</v>
       </c>
@@ -947,7 +946,7 @@
       <c r="J5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K5" s="2"/>
+      <c r="K5" s="4"/>
       <c r="L5" s="2" t="s">
         <v>20</v>
       </c>
@@ -983,7 +982,7 @@
       <c r="J6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" s="4"/>
       <c r="L6" s="2" t="s">
         <v>45</v>
       </c>
@@ -1019,7 +1018,7 @@
       <c r="J7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="2"/>
+      <c r="K7" s="4"/>
       <c r="L7" s="2" t="s">
         <v>20</v>
       </c>
@@ -1055,7 +1054,7 @@
       <c r="J8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="4" t="s">
         <v>56</v>
       </c>
       <c r="L8" s="2" t="s">
@@ -1093,7 +1092,7 @@
       <c r="J9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="2"/>
+      <c r="K9" s="4"/>
       <c r="L9" s="2" t="s">
         <v>20</v>
       </c>
@@ -1129,7 +1128,7 @@
       <c r="J10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="4" t="s">
         <v>67</v>
       </c>
       <c r="L10" s="2" t="s">
@@ -1164,10 +1163,10 @@
       <c r="I11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L11" s="2" t="s">
@@ -1205,7 +1204,7 @@
       <c r="J12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="K12" s="4" t="s">
         <v>79</v>
       </c>
       <c r="L12" s="2" t="s">
@@ -1243,7 +1242,7 @@
       <c r="J13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="2"/>
+      <c r="K13" s="4"/>
       <c r="L13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1279,7 +1278,7 @@
       <c r="J14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K14" s="2"/>
+      <c r="K14" s="4"/>
       <c r="L14" s="2" t="s">
         <v>20</v>
       </c>
@@ -1315,7 +1314,7 @@
       <c r="J15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="2"/>
+      <c r="K15" s="4"/>
       <c r="L15" s="2" t="s">
         <v>45</v>
       </c>
@@ -1351,7 +1350,7 @@
       <c r="J16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="2"/>
+      <c r="K16" s="4"/>
       <c r="L16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1387,7 +1386,7 @@
       <c r="J17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="K17" s="4" t="s">
         <v>102</v>
       </c>
       <c r="L17" s="2" t="s">
@@ -1425,7 +1424,7 @@
       <c r="J18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="K18" s="4" t="s">
         <v>105</v>
       </c>
       <c r="L18" s="2" t="s">
@@ -1463,7 +1462,7 @@
       <c r="J19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K19" s="2"/>
+      <c r="K19" s="4"/>
       <c r="L19" s="2" t="s">
         <v>20</v>
       </c>
@@ -1499,14 +1498,14 @@
       <c r="J20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="K20" s="4" t="s">
         <v>115</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>116</v>
       </c>
@@ -1537,14 +1536,14 @@
       <c r="J21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="K21" s="4" t="s">
         <v>120</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>121</v>
       </c>

</xml_diff>